<commit_message>
tag06 mit HA gespeichert
</commit_message>
<xml_diff>
--- a/src/main/java/tag05/aufgabe/A_L1.xlsx
+++ b/src/main/java/tag05/aufgabe/A_L1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahaas8\IdeaProjects\TF_US_PM1\src\main\java\tag05\aufgabe\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B6E9A9-E941-438F-A82F-E77787A4F699}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB362D77-60FA-4247-A413-6CED299B0D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2610" windowWidth="21600" windowHeight="11295" xr2:uid="{78E59CFC-51CD-44E2-918C-96DBDC140821}"/>
+    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{78E59CFC-51CD-44E2-918C-96DBDC140821}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Funktionalität</t>
   </si>
@@ -57,6 +57,15 @@
   </si>
   <si>
     <t>Anbieter3</t>
+  </si>
+  <si>
+    <t>Mit Priorität</t>
+  </si>
+  <si>
+    <t>Platz</t>
+  </si>
+  <si>
+    <t>Gewichtung</t>
   </si>
 </sst>
 </file>
@@ -110,11 +119,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -449,91 +471,133 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CA056CF-E941-47A5-A8F6-C7A8F0BAF630}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="5">
         <v>3</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="6">
         <v>4</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="7">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="5">
         <v>5</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="6">
         <v>3</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="7">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="5">
         <v>4</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="6">
         <v>6</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="7">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" s="8">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>2</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="6">
         <v>3</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="7">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
-        <f>SUM(B2:B5)</f>
-        <v>14</v>
-      </c>
-      <c r="C6" s="1">
-        <f t="shared" ref="C6:D6" si="0">SUM(C2:C5)</f>
-        <v>16</v>
-      </c>
-      <c r="D6" s="2">
+      <c r="E5" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <f>(B2*$E$2) + (B3*$E$3) + (B4*$E$4) + (B5*$E$5)</f>
+        <v>390</v>
+      </c>
+      <c r="C8">
+        <f t="shared" ref="C8:D8" si="0">(C2*$E$2) + (C3*$E$3) + (C4*$E$4) + (C5*$E$5)</f>
+        <v>440</v>
+      </c>
+      <c r="D8">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>350</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>2</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>